<commit_message>
Make M06 artifacts reproducible and tighten audit key
Co-authored-by: shaseaver25 <shannon@tailoredu.org>
</commit_message>
<xml_diff>
--- a/teaching-pack/10-M06-alarm-audit/M06-gauge-audit-and-handoff.xlsx
+++ b/teaching-pack/10-M06-alarm-audit/M06-gauge-audit-and-handoff.xlsx
@@ -1071,7 +1071,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1147,7 +1147,7 @@
       <c r="B8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>RETAIN THIS RECORD</t>
         </is>
@@ -1157,9 +1157,6 @@
           <t>This February file returns later in the project.</t>
         </is>
       </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:B9"/>

</xml_diff>